<commit_message>
New ontologies: brcomp and bmap
</commit_message>
<xml_diff>
--- a/data/Ontologies_forRepo.xlsx
+++ b/data/Ontologies_forRepo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CH157"/>
+  <dimension ref="A1:CH159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1850,12 +1850,12 @@
       <c r="BM5" t="inlineStr"/>
       <c r="BN5" t="inlineStr">
         <is>
-          <t>n051fc69bd461486ca10f9025fc99477ab1</t>
+          <t>n37add634c1ab498cb948a7fa86936747b1</t>
         </is>
       </c>
       <c r="BO5" t="inlineStr">
         <is>
-          <t>n051fc69bd461486ca10f9025fc99477ab1</t>
+          <t>n37add634c1ab498cb948a7fa86936747b1</t>
         </is>
       </c>
       <c r="BP5" t="inlineStr"/>
@@ -2109,12 +2109,12 @@
       </c>
       <c r="BN6" t="inlineStr">
         <is>
-          <t>nebf49109c8634b9d8df5721e35341f53b1</t>
+          <t>n3d9f1dd166da442da814fc23fa4b1084b1</t>
         </is>
       </c>
       <c r="BO6" t="inlineStr">
         <is>
-          <t>nebf49109c8634b9d8df5721e35341f53b1</t>
+          <t>n3d9f1dd166da442da814fc23fa4b1084b1</t>
         </is>
       </c>
       <c r="BP6" t="inlineStr"/>
@@ -3022,12 +3022,12 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>brot, bot, reloc, infraspatialot, bcoremedia</t>
+          <t>brot, bot, reloc, infraspatialot, bcoremedia, bmat</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>brot, bot, reloc, infraspatialot, bcoremedia</t>
+          <t>brot, bot, reloc, infraspatialot, bcoremedia, bmat</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
@@ -3037,12 +3037,12 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>dc, dcterms, bibo, vann, foaf, schema, bmat, brcomp</t>
+          <t>dc, dcterms, bibo, vann, foaf, schema, brcomp</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>dc, dcterms, bibo, vann, foaf, schema, bmat, brcomp</t>
+          <t>dc, dcterms, bibo, vann, foaf, schema, brcomp</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr"/>
@@ -3196,7 +3196,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://w3id.org/bcore/comp</t>
+          <t>https://w3id.org/bcore/comp#</t>
         </is>
       </c>
       <c r="B11" t="b">
@@ -3486,7 +3486,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://w3id.org/bcore/infra</t>
+          <t>https://w3id.org/bcore/infra#</t>
         </is>
       </c>
       <c r="B12" t="b">
@@ -3762,7 +3762,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://w3id.org/bcore/mat</t>
+          <t>https://w3id.org/bcore/mat#</t>
         </is>
       </c>
       <c r="B13" t="b">
@@ -3865,11 +3865,19 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>bcore</t>
-        </is>
-      </c>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
+          <t>bcore, bmat</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>bmat</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>bmat</t>
+        </is>
+      </c>
       <c r="AA13" t="inlineStr">
         <is>
           <t>vann, foaf, schema, bibo</t>
@@ -3877,12 +3885,12 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>bmat, dc, dcterms, bibo, vann, foaf, schema</t>
+          <t>dc, dcterms, bibo, vann, foaf, schema</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>bmat, dc, dcterms, bibo, vann, foaf, schema</t>
+          <t>dc, dcterms, bibo, vann, foaf, schema</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr"/>
@@ -4014,13 +4022,13 @@
         <v>1</v>
       </c>
       <c r="BZ13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CA13" t="b">
         <v>0</v>
       </c>
       <c r="CB13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CC13" t="n">
         <v>2</v>
@@ -4044,7 +4052,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://w3id.org/bcore/media</t>
+          <t>https://w3id.org/bcore/media#</t>
         </is>
       </c>
       <c r="B14" t="b">
@@ -4218,10 +4226,10 @@
       </c>
       <c r="AS14" t="inlineStr"/>
       <c r="AT14" t="n">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
       <c r="AU14" t="n">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
       <c r="AV14" t="inlineStr"/>
       <c r="AW14" t="inlineStr"/>
@@ -4330,7 +4338,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://w3id.org/bcore/zones</t>
+          <t>https://w3id.org/bcore/zones#</t>
         </is>
       </c>
       <c r="B15" t="b">
@@ -5561,12 +5569,12 @@
       <c r="BM19" t="inlineStr"/>
       <c r="BN19" t="inlineStr">
         <is>
-          <t>nc29cda6e1fb6476eae76fd998bccf4e6b1</t>
+          <t>ne9049731d41245fdb9604b40945f820fb1</t>
         </is>
       </c>
       <c r="BO19" t="inlineStr">
         <is>
-          <t>nc29cda6e1fb6476eae76fd998bccf4e6b1</t>
+          <t>ne9049731d41245fdb9604b40945f820fb1</t>
         </is>
       </c>
       <c r="BP19" t="inlineStr"/>
@@ -7537,12 +7545,12 @@
       <c r="BM27" t="inlineStr"/>
       <c r="BN27" t="inlineStr">
         <is>
-          <t>n186cd50b1ad349888714233d7ee55eb9b8, n186cd50b1ad349888714233d7ee55eb9b9, n186cd50b1ad349888714233d7ee55eb9b10, n186cd50b1ad349888714233d7ee55eb9b11</t>
+          <t>n93b9729fe41b4116b4b844a34fd6e556b8, n93b9729fe41b4116b4b844a34fd6e556b9, n93b9729fe41b4116b4b844a34fd6e556b10, n93b9729fe41b4116b4b844a34fd6e556b11</t>
         </is>
       </c>
       <c r="BO27" t="inlineStr">
         <is>
-          <t>n186cd50b1ad349888714233d7ee55eb9b8, n186cd50b1ad349888714233d7ee55eb9b9, n186cd50b1ad349888714233d7ee55eb9b10, n186cd50b1ad349888714233d7ee55eb9b11</t>
+          <t>n93b9729fe41b4116b4b844a34fd6e556b8, n93b9729fe41b4116b4b844a34fd6e556b9, n93b9729fe41b4116b4b844a34fd6e556b10, n93b9729fe41b4116b4b844a34fd6e556b11</t>
         </is>
       </c>
       <c r="BP27" t="inlineStr"/>
@@ -7817,22 +7825,22 @@
       </c>
       <c r="BN28" t="inlineStr">
         <is>
-          <t>n5d86b0eeebf648efbe7729fb2cf897a1b7274</t>
+          <t>n54ed29e592f049fa9c635904677b4703b7274</t>
         </is>
       </c>
       <c r="BO28" t="inlineStr">
         <is>
-          <t>n5d86b0eeebf648efbe7729fb2cf897a1b7274</t>
+          <t>n54ed29e592f049fa9c635904677b4703b7274</t>
         </is>
       </c>
       <c r="BP28" t="inlineStr">
         <is>
-          <t>n5d86b0eeebf648efbe7729fb2cf897a1b7276</t>
+          <t>n54ed29e592f049fa9c635904677b4703b7276</t>
         </is>
       </c>
       <c r="BQ28" t="inlineStr">
         <is>
-          <t>n5d86b0eeebf648efbe7729fb2cf897a1b7276</t>
+          <t>n54ed29e592f049fa9c635904677b4703b7276</t>
         </is>
       </c>
       <c r="BR28" t="inlineStr">
@@ -8036,12 +8044,12 @@
       </c>
       <c r="AQ29" t="inlineStr">
         <is>
-          <t>bcore, bcorecomp, bcoremedia, bedo</t>
+          <t>bcore, bcorecomp, bcoremedia, bedo, bmat, brcomp</t>
         </is>
       </c>
       <c r="AR29" t="inlineStr">
         <is>
-          <t>bcore, bcorecomp, bcoremedia, bedo</t>
+          <t>bcore, bcorecomp, bcoremedia, bedo, bmat, brcomp</t>
         </is>
       </c>
       <c r="AS29" t="inlineStr"/>
@@ -8091,12 +8099,12 @@
       <c r="BM29" t="inlineStr"/>
       <c r="BN29" t="inlineStr">
         <is>
-          <t>n853daf604e094e68b5b4eda554efe446b1, n853daf604e094e68b5b4eda554efe446b2</t>
+          <t>nc73f03e7dd51442c9baea22cf394a7f6b1, nc73f03e7dd51442c9baea22cf394a7f6b2</t>
         </is>
       </c>
       <c r="BO29" t="inlineStr">
         <is>
-          <t>n853daf604e094e68b5b4eda554efe446b1, n853daf604e094e68b5b4eda554efe446b2</t>
+          <t>nc73f03e7dd51442c9baea22cf394a7f6b1, nc73f03e7dd51442c9baea22cf394a7f6b2</t>
         </is>
       </c>
       <c r="BP29" t="inlineStr"/>
@@ -8837,12 +8845,12 @@
       <c r="BM32" t="inlineStr"/>
       <c r="BN32" t="inlineStr">
         <is>
-          <t>nd11198aa82554de5b40d2cf014d4d25fb1</t>
+          <t>n4a5b99de31cc418f8e6b771499ab9653b1</t>
         </is>
       </c>
       <c r="BO32" t="inlineStr">
         <is>
-          <t>nd11198aa82554de5b40d2cf014d4d25fb1</t>
+          <t>n4a5b99de31cc418f8e6b771499ab9653b1</t>
         </is>
       </c>
       <c r="BP32" t="inlineStr"/>
@@ -9537,12 +9545,12 @@
       <c r="BM35" t="inlineStr"/>
       <c r="BN35" t="inlineStr">
         <is>
-          <t>n15827cb90fce43df8294d98f7b1a69d0b3, n15827cb90fce43df8294d98f7b1a69d0b4</t>
+          <t>n5253fd3235204cb19cc4c87c2fa4b5b3b3, n5253fd3235204cb19cc4c87c2fa4b5b3b4</t>
         </is>
       </c>
       <c r="BO35" t="inlineStr">
         <is>
-          <t>n15827cb90fce43df8294d98f7b1a69d0b3, n15827cb90fce43df8294d98f7b1a69d0b4</t>
+          <t>n5253fd3235204cb19cc4c87c2fa4b5b3b3, n5253fd3235204cb19cc4c87c2fa4b5b3b4</t>
         </is>
       </c>
       <c r="BP35" t="inlineStr"/>
@@ -10015,12 +10023,12 @@
       </c>
       <c r="BN37" t="inlineStr">
         <is>
-          <t>nb19a3959f4b54eeaa5181b80535272c6b1</t>
+          <t>n88ed93e1111644cd99d04863357c6acbb1</t>
         </is>
       </c>
       <c r="BO37" t="inlineStr">
         <is>
-          <t>nb19a3959f4b54eeaa5181b80535272c6b1</t>
+          <t>n88ed93e1111644cd99d04863357c6acbb1</t>
         </is>
       </c>
       <c r="BP37" t="inlineStr"/>
@@ -10311,12 +10319,12 @@
       <c r="BM38" t="inlineStr"/>
       <c r="BN38" t="inlineStr">
         <is>
-          <t>n4f3d3308f60d48e78aa7729ed0028a2fb3, n4f3d3308f60d48e78aa7729ed0028a2fb4</t>
+          <t>nca082b3b2a4e401eb84be56bedf36108b3, nca082b3b2a4e401eb84be56bedf36108b4</t>
         </is>
       </c>
       <c r="BO38" t="inlineStr">
         <is>
-          <t>n4f3d3308f60d48e78aa7729ed0028a2fb3, n4f3d3308f60d48e78aa7729ed0028a2fb4</t>
+          <t>nca082b3b2a4e401eb84be56bedf36108b3, nca082b3b2a4e401eb84be56bedf36108b4</t>
         </is>
       </c>
       <c r="BP38" t="inlineStr"/>
@@ -10607,12 +10615,12 @@
       <c r="BM39" t="inlineStr"/>
       <c r="BN39" t="inlineStr">
         <is>
-          <t>n6d33c850967c40959b1027a156eb6518b3, n6d33c850967c40959b1027a156eb6518b4</t>
+          <t>n40970c4c58ef47b5afb92474f38138a6b3, n40970c4c58ef47b5afb92474f38138a6b4</t>
         </is>
       </c>
       <c r="BO39" t="inlineStr">
         <is>
-          <t>n6d33c850967c40959b1027a156eb6518b3, n6d33c850967c40959b1027a156eb6518b4</t>
+          <t>n40970c4c58ef47b5afb92474f38138a6b3, n40970c4c58ef47b5afb92474f38138a6b4</t>
         </is>
       </c>
       <c r="BP39" t="inlineStr"/>
@@ -10896,12 +10904,12 @@
       <c r="BM40" t="inlineStr"/>
       <c r="BN40" t="inlineStr">
         <is>
-          <t>ne9ed3b9aecaf4ed08aa5ba1afeca9404b1</t>
+          <t>n385d58e316724bf8bfc0822536fd9769b1</t>
         </is>
       </c>
       <c r="BO40" t="inlineStr">
         <is>
-          <t>ne9ed3b9aecaf4ed08aa5ba1afeca9404b1</t>
+          <t>n385d58e316724bf8bfc0822536fd9769b1</t>
         </is>
       </c>
       <c r="BP40" t="inlineStr"/>
@@ -11177,22 +11185,22 @@
       <c r="BM41" t="inlineStr"/>
       <c r="BN41" t="inlineStr">
         <is>
-          <t>n2df3c4579f3d402b99b607e66b2ddad1b1</t>
+          <t>nabd7b40594274f8fa647dfe713a48eaeb1</t>
         </is>
       </c>
       <c r="BO41" t="inlineStr">
         <is>
-          <t>n2df3c4579f3d402b99b607e66b2ddad1b1</t>
+          <t>nabd7b40594274f8fa647dfe713a48eaeb1</t>
         </is>
       </c>
       <c r="BP41" t="inlineStr">
         <is>
-          <t>n2df3c4579f3d402b99b607e66b2ddad1b3</t>
+          <t>nabd7b40594274f8fa647dfe713a48eaeb3</t>
         </is>
       </c>
       <c r="BQ41" t="inlineStr">
         <is>
-          <t>n2df3c4579f3d402b99b607e66b2ddad1b3</t>
+          <t>nabd7b40594274f8fa647dfe713a48eaeb3</t>
         </is>
       </c>
       <c r="BR41" t="inlineStr">
@@ -16278,12 +16286,12 @@
       </c>
       <c r="BN60" t="inlineStr">
         <is>
-          <t>na5a8b9ed6406407a9dca26b809994123b1, https://www.researchgate.net/profile/Mathias_Bonduel</t>
+          <t>n473d206037a24fb8b144c97a9f119d93b1, https://www.researchgate.net/profile/Mathias_Bonduel</t>
         </is>
       </c>
       <c r="BO60" t="inlineStr">
         <is>
-          <t>na5a8b9ed6406407a9dca26b809994123b1, https://www.researchgate.net/profile/Mathias_Bonduel</t>
+          <t>n473d206037a24fb8b144c97a9f119d93b1, https://www.researchgate.net/profile/Mathias_Bonduel</t>
         </is>
       </c>
       <c r="BP60" t="inlineStr"/>
@@ -20867,12 +20875,12 @@
       </c>
       <c r="BP78" t="inlineStr">
         <is>
-          <t>nc65800fa3f144939994cc46e61376703b1</t>
+          <t>n189b8926b4ba49ea8f359a264ca0090db1</t>
         </is>
       </c>
       <c r="BQ78" t="inlineStr">
         <is>
-          <t>nc65800fa3f144939994cc46e61376703b1</t>
+          <t>n189b8926b4ba49ea8f359a264ca0090db1</t>
         </is>
       </c>
       <c r="BR78" t="inlineStr">
@@ -22161,22 +22169,22 @@
       <c r="BM83" t="inlineStr"/>
       <c r="BN83" t="inlineStr">
         <is>
-          <t>nd9eb571ee4414d3ea9587e9a1ef9f7c9b1</t>
+          <t>n719fb6e75be843b6b442662d72ffc7a7b1</t>
         </is>
       </c>
       <c r="BO83" t="inlineStr">
         <is>
-          <t>nd9eb571ee4414d3ea9587e9a1ef9f7c9b1</t>
+          <t>n719fb6e75be843b6b442662d72ffc7a7b1</t>
         </is>
       </c>
       <c r="BP83" t="inlineStr">
         <is>
-          <t>nd9eb571ee4414d3ea9587e9a1ef9f7c9b3</t>
+          <t>n719fb6e75be843b6b442662d72ffc7a7b3</t>
         </is>
       </c>
       <c r="BQ83" t="inlineStr">
         <is>
-          <t>nd9eb571ee4414d3ea9587e9a1ef9f7c9b3</t>
+          <t>n719fb6e75be843b6b442662d72ffc7a7b3</t>
         </is>
       </c>
       <c r="BR83" t="inlineStr">
@@ -22949,12 +22957,12 @@
       <c r="BM86" t="inlineStr"/>
       <c r="BN86" t="inlineStr">
         <is>
-          <t>n0b6d7c418c694dfa8f53bf9eb5151348b1, n0b6d7c418c694dfa8f53bf9eb5151348b2</t>
+          <t>n3ab4571434c64d8cb3467a5f242dc0c4b1, n3ab4571434c64d8cb3467a5f242dc0c4b2</t>
         </is>
       </c>
       <c r="BO86" t="inlineStr">
         <is>
-          <t>n0b6d7c418c694dfa8f53bf9eb5151348b1, n0b6d7c418c694dfa8f53bf9eb5151348b2</t>
+          <t>n3ab4571434c64d8cb3467a5f242dc0c4b1, n3ab4571434c64d8cb3467a5f242dc0c4b2</t>
         </is>
       </c>
       <c r="BP86" t="inlineStr"/>
@@ -24074,22 +24082,22 @@
       <c r="BM90" t="inlineStr"/>
       <c r="BN90" t="inlineStr">
         <is>
-          <t>n08709a39882e49a0bc6210aeb2ea7356b3, n08709a39882e49a0bc6210aeb2ea7356b5</t>
+          <t>n2e68452f92ab46509affcd652bbe7005b3, n2e68452f92ab46509affcd652bbe7005b5</t>
         </is>
       </c>
       <c r="BO90" t="inlineStr">
         <is>
-          <t>n08709a39882e49a0bc6210aeb2ea7356b3, n08709a39882e49a0bc6210aeb2ea7356b5</t>
+          <t>n2e68452f92ab46509affcd652bbe7005b3, n2e68452f92ab46509affcd652bbe7005b5</t>
         </is>
       </c>
       <c r="BP90" t="inlineStr">
         <is>
-          <t>n08709a39882e49a0bc6210aeb2ea7356b7</t>
+          <t>n2e68452f92ab46509affcd652bbe7005b7</t>
         </is>
       </c>
       <c r="BQ90" t="inlineStr">
         <is>
-          <t>n08709a39882e49a0bc6210aeb2ea7356b7</t>
+          <t>n2e68452f92ab46509affcd652bbe7005b7</t>
         </is>
       </c>
       <c r="BR90" t="inlineStr">
@@ -25063,22 +25071,22 @@
       <c r="BM94" t="inlineStr"/>
       <c r="BN94" t="inlineStr">
         <is>
-          <t>nd90612088c7d4a9e94f99d87870a61e3b3, nd90612088c7d4a9e94f99d87870a61e3b5</t>
+          <t>n9c50b06e351a4379b54de82cc3ad0bf1b3, n9c50b06e351a4379b54de82cc3ad0bf1b5</t>
         </is>
       </c>
       <c r="BO94" t="inlineStr">
         <is>
-          <t>nd90612088c7d4a9e94f99d87870a61e3b3, nd90612088c7d4a9e94f99d87870a61e3b5</t>
+          <t>n9c50b06e351a4379b54de82cc3ad0bf1b3, n9c50b06e351a4379b54de82cc3ad0bf1b5</t>
         </is>
       </c>
       <c r="BP94" t="inlineStr">
         <is>
-          <t>nd90612088c7d4a9e94f99d87870a61e3b7</t>
+          <t>n9c50b06e351a4379b54de82cc3ad0bf1b7</t>
         </is>
       </c>
       <c r="BQ94" t="inlineStr">
         <is>
-          <t>nd90612088c7d4a9e94f99d87870a61e3b7</t>
+          <t>n9c50b06e351a4379b54de82cc3ad0bf1b7</t>
         </is>
       </c>
       <c r="BR94" t="inlineStr">
@@ -25897,12 +25905,12 @@
       </c>
       <c r="BN97" t="inlineStr">
         <is>
-          <t>ndb4ebdd8bdef41d6b41faaad3c8d614cb1</t>
+          <t>n1d457ef97f4541b991e774e0ef77205ab1</t>
         </is>
       </c>
       <c r="BO97" t="inlineStr">
         <is>
-          <t>ndb4ebdd8bdef41d6b41faaad3c8d614cb1</t>
+          <t>n1d457ef97f4541b991e774e0ef77205ab1</t>
         </is>
       </c>
       <c r="BP97" t="inlineStr"/>
@@ -28791,12 +28799,12 @@
       <c r="BM109" t="inlineStr"/>
       <c r="BN109" t="inlineStr">
         <is>
-          <t>nd9ff4291497b4f738baedb5ef335fe73b1, nd9ff4291497b4f738baedb5ef335fe73b2</t>
+          <t>n0c7153e579c5459ba422335ff4d7a272b1, n0c7153e579c5459ba422335ff4d7a272b2</t>
         </is>
       </c>
       <c r="BO109" t="inlineStr">
         <is>
-          <t>nd9ff4291497b4f738baedb5ef335fe73b1, nd9ff4291497b4f738baedb5ef335fe73b2</t>
+          <t>n0c7153e579c5459ba422335ff4d7a272b1, n0c7153e579c5459ba422335ff4d7a272b2</t>
         </is>
       </c>
       <c r="BP109" t="inlineStr"/>
@@ -37867,12 +37875,12 @@
       <c r="BM142" t="inlineStr"/>
       <c r="BN142" t="inlineStr">
         <is>
-          <t>n33fcc512c49c4ff6b34babb58299cf75b1</t>
+          <t>n7f7d721c4294429fa9e60aa20d8a148eb1</t>
         </is>
       </c>
       <c r="BO142" t="inlineStr">
         <is>
-          <t>n33fcc512c49c4ff6b34babb58299cf75b1</t>
+          <t>n7f7d721c4294429fa9e60aa20d8a148eb1</t>
         </is>
       </c>
       <c r="BP142" t="inlineStr"/>
@@ -38149,12 +38157,12 @@
       <c r="BM143" t="inlineStr"/>
       <c r="BN143" t="inlineStr">
         <is>
-          <t>n32237aee44da4072b37e5cfaaf63d857b1</t>
+          <t>nf3a95ff3b0084e419923e556eef9feb4b1</t>
         </is>
       </c>
       <c r="BO143" t="inlineStr">
         <is>
-          <t>n32237aee44da4072b37e5cfaaf63d857b1</t>
+          <t>nf3a95ff3b0084e419923e556eef9feb4b1</t>
         </is>
       </c>
       <c r="BP143" t="inlineStr"/>
@@ -38702,22 +38710,22 @@
       </c>
       <c r="BN145" t="inlineStr">
         <is>
-          <t>n3370fd46a4c74366abb405c451ee2ebdb1, n3370fd46a4c74366abb405c451ee2ebdb3, n3370fd46a4c74366abb405c451ee2ebdb5, n3370fd46a4c74366abb405c451ee2ebdb7</t>
+          <t>nc381259b2c1e4a4585fe161174b68472b1, nc381259b2c1e4a4585fe161174b68472b3, nc381259b2c1e4a4585fe161174b68472b5, nc381259b2c1e4a4585fe161174b68472b7</t>
         </is>
       </c>
       <c r="BO145" t="inlineStr">
         <is>
-          <t>n3370fd46a4c74366abb405c451ee2ebdb1, n3370fd46a4c74366abb405c451ee2ebdb3, n3370fd46a4c74366abb405c451ee2ebdb5, n3370fd46a4c74366abb405c451ee2ebdb7</t>
+          <t>nc381259b2c1e4a4585fe161174b68472b1, nc381259b2c1e4a4585fe161174b68472b3, nc381259b2c1e4a4585fe161174b68472b5, nc381259b2c1e4a4585fe161174b68472b7</t>
         </is>
       </c>
       <c r="BP145" t="inlineStr">
         <is>
-          <t>n3370fd46a4c74366abb405c451ee2ebdb9</t>
+          <t>nc381259b2c1e4a4585fe161174b68472b9</t>
         </is>
       </c>
       <c r="BQ145" t="inlineStr">
         <is>
-          <t>n3370fd46a4c74366abb405c451ee2ebdb9</t>
+          <t>nc381259b2c1e4a4585fe161174b68472b9</t>
         </is>
       </c>
       <c r="BR145" t="inlineStr">
@@ -41517,6 +41525,472 @@
         <v>1</v>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>https://w3id.org/bmat</t>
+        </is>
+      </c>
+      <c r="B158" t="b">
+        <v>1</v>
+      </c>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>bmat</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>bmat</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>bmat</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>BMAT - Ontology for defining building materials.</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr"/>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>BMAT - Ontology for defining building materials.</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Ontology for defining building materials.
+The suggested prefix for the BMAT namespace is bmat
+It is recommended to use BMAT in conjunction with BROT for defining a bridge construction and its aggregated components.</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>Ontology for defining building materials.
+The suggested prefix for the BMAT namespace is bmat
+It is recommended to use BMAT in conjunction with BROT for defining a bridge construction and its aggregated components.</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr"/>
+      <c r="N158" t="inlineStr"/>
+      <c r="O158" t="inlineStr"/>
+      <c r="P158" t="inlineStr"/>
+      <c r="Q158" t="inlineStr"/>
+      <c r="R158" t="inlineStr"/>
+      <c r="S158" t="inlineStr"/>
+      <c r="T158" t="inlineStr"/>
+      <c r="U158" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="V158" t="inlineStr"/>
+      <c r="W158" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="X158" t="inlineStr">
+        <is>
+          <t>brcomp, brot</t>
+        </is>
+      </c>
+      <c r="Y158" t="inlineStr">
+        <is>
+          <t>brot</t>
+        </is>
+      </c>
+      <c r="Z158" t="inlineStr">
+        <is>
+          <t>brot</t>
+        </is>
+      </c>
+      <c r="AA158" t="inlineStr">
+        <is>
+          <t>schema, foaf, vann, cd</t>
+        </is>
+      </c>
+      <c r="AB158" t="inlineStr">
+        <is>
+          <t>foaf, vann, schema, brcomp</t>
+        </is>
+      </c>
+      <c r="AC158" t="inlineStr">
+        <is>
+          <t>foaf, vann, schema, brcomp</t>
+        </is>
+      </c>
+      <c r="AD158" t="inlineStr"/>
+      <c r="AE158" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF158" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG158" t="inlineStr"/>
+      <c r="AH158" t="inlineStr"/>
+      <c r="AI158" t="inlineStr"/>
+      <c r="AJ158" t="inlineStr"/>
+      <c r="AK158" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL158" t="b">
+        <v>1</v>
+      </c>
+      <c r="AM158" t="n">
+        <v>100</v>
+      </c>
+      <c r="AN158" t="inlineStr"/>
+      <c r="AO158" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP158" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ158" t="inlineStr">
+        <is>
+          <t>bcore, bcoremat</t>
+        </is>
+      </c>
+      <c r="AR158" t="inlineStr">
+        <is>
+          <t>bcore, bcoremat</t>
+        </is>
+      </c>
+      <c r="AS158" t="inlineStr"/>
+      <c r="AT158" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AU158" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AV158" t="inlineStr"/>
+      <c r="AW158" t="inlineStr"/>
+      <c r="AX158" t="inlineStr"/>
+      <c r="AY158" t="b">
+        <v>0</v>
+      </c>
+      <c r="AZ158" t="inlineStr"/>
+      <c r="BA158" t="b">
+        <v>0</v>
+      </c>
+      <c r="BB158" t="inlineStr"/>
+      <c r="BC158" t="inlineStr"/>
+      <c r="BD158" t="inlineStr"/>
+      <c r="BE158" t="inlineStr">
+        <is>
+          <t>https://alhakam.github.io/bmat/</t>
+        </is>
+      </c>
+      <c r="BF158" t="inlineStr"/>
+      <c r="BG158" t="inlineStr">
+        <is>
+          <t>https://alhakam.github.io/bmat/</t>
+        </is>
+      </c>
+      <c r="BH158" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="BI158" t="inlineStr"/>
+      <c r="BJ158" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="BK158" t="inlineStr"/>
+      <c r="BL158" t="inlineStr"/>
+      <c r="BM158" t="inlineStr"/>
+      <c r="BN158" t="inlineStr"/>
+      <c r="BO158" t="inlineStr"/>
+      <c r="BP158" t="inlineStr"/>
+      <c r="BQ158" t="inlineStr"/>
+      <c r="BR158" t="inlineStr">
+        <is>
+          <t>{owl: http://www.w3.org/2002/07/owl#}, {rdf: http://www.w3.org/1999/02/22-rdf-syntax-ns#}, {xsd: http://www.w3.org/2001/XMLSchema#}, {brot: https://w3id.org/brot#}, {foaf: http://xmlns.com/foaf/0.1/}, {rdfs: http://www.w3.org/2000/01/rdf-schema#}, {vann: http://purl.org/vocab/vann/}, {schema: http://schema.org/#}, {brcomp: https://w3id.org/brcomp#}, {None: http://purl.org/dc/}</t>
+        </is>
+      </c>
+      <c r="BS158" t="n">
+        <v>7</v>
+      </c>
+      <c r="BT158" t="n">
+        <v>7</v>
+      </c>
+      <c r="BU158" t="n">
+        <v>26</v>
+      </c>
+      <c r="BV158" t="n">
+        <v>26</v>
+      </c>
+      <c r="BW158" t="n">
+        <v>2</v>
+      </c>
+      <c r="BX158" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY158" t="b">
+        <v>1</v>
+      </c>
+      <c r="BZ158" t="b">
+        <v>1</v>
+      </c>
+      <c r="CA158" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB158" t="n">
+        <v>2</v>
+      </c>
+      <c r="CC158" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD158" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE158" t="b">
+        <v>0</v>
+      </c>
+      <c r="CF158" t="b">
+        <v>1</v>
+      </c>
+      <c r="CG158" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH158" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>https://w3id.org//brcomp#</t>
+        </is>
+      </c>
+      <c r="B159" t="b">
+        <v>1</v>
+      </c>
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>brcomp</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>brcomp</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>brcomp</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Bridge Components (BRCOMP)</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Bridge Components (BRCOMP)</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>he ontology for Bridge Components (BRCOMP) allows the further classification of Bridge Elements defined in BROT. Furthermore, additional domain-specific data properties can be assigned to the instances of Bridge Element.
+The namespace for BRCOMP terms is https://w3id.org//brcomp#
+The suggested prefix for the BRCOMP namespace is brcomp
+It is recommended to use BRCOMP in conjunction with BROT for defining a bridge construction and its aggregated components.</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr"/>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>he ontology for Bridge Components (BRCOMP) allows the further classification of Bridge Elements defined in BROT. Furthermore, additional domain-specific data properties can be assigned to the instances of Bridge Element.
+The namespace for BRCOMP terms is https://w3id.org//brcomp#
+The suggested prefix for the BRCOMP namespace is brcomp
+It is recommended to use BRCOMP in conjunction with BROT for defining a bridge construction and its aggregated components.</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr"/>
+      <c r="N159" t="inlineStr"/>
+      <c r="O159" t="inlineStr"/>
+      <c r="P159" t="inlineStr"/>
+      <c r="Q159" t="inlineStr"/>
+      <c r="R159" t="inlineStr"/>
+      <c r="S159" t="inlineStr"/>
+      <c r="T159" t="inlineStr"/>
+      <c r="U159" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="V159" t="inlineStr"/>
+      <c r="W159" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="X159" t="inlineStr">
+        <is>
+          <t>brot</t>
+        </is>
+      </c>
+      <c r="Y159" t="inlineStr">
+        <is>
+          <t>brot</t>
+        </is>
+      </c>
+      <c r="Z159" t="inlineStr">
+        <is>
+          <t>brot</t>
+        </is>
+      </c>
+      <c r="AA159" t="inlineStr">
+        <is>
+          <t>vann, foaf, dc</t>
+        </is>
+      </c>
+      <c r="AB159" t="inlineStr">
+        <is>
+          <t>foaf, vann</t>
+        </is>
+      </c>
+      <c r="AC159" t="inlineStr">
+        <is>
+          <t>foaf, vann</t>
+        </is>
+      </c>
+      <c r="AD159" t="inlineStr"/>
+      <c r="AE159" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF159" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG159" t="inlineStr"/>
+      <c r="AH159" t="inlineStr"/>
+      <c r="AI159" t="inlineStr"/>
+      <c r="AJ159" t="inlineStr"/>
+      <c r="AK159" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL159" t="b">
+        <v>1</v>
+      </c>
+      <c r="AM159" t="n">
+        <v>98.7</v>
+      </c>
+      <c r="AN159" t="inlineStr"/>
+      <c r="AO159" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP159" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ159" t="inlineStr"/>
+      <c r="AR159" t="inlineStr"/>
+      <c r="AS159" t="inlineStr"/>
+      <c r="AT159" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AU159" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AV159" t="inlineStr"/>
+      <c r="AW159" t="inlineStr"/>
+      <c r="AX159" t="inlineStr"/>
+      <c r="AY159" t="b">
+        <v>0</v>
+      </c>
+      <c r="AZ159" t="inlineStr"/>
+      <c r="BA159" t="b">
+        <v>0</v>
+      </c>
+      <c r="BB159" t="inlineStr"/>
+      <c r="BC159" t="inlineStr"/>
+      <c r="BD159" t="inlineStr"/>
+      <c r="BE159" t="inlineStr">
+        <is>
+          <t>https://alhakam.github.io/brcomp/</t>
+        </is>
+      </c>
+      <c r="BF159" t="inlineStr"/>
+      <c r="BG159" t="inlineStr">
+        <is>
+          <t>https://alhakam.github.io/brcomp/</t>
+        </is>
+      </c>
+      <c r="BH159" t="inlineStr">
+        <is>
+          <t>BE Product (Infrastructure)</t>
+        </is>
+      </c>
+      <c r="BI159" t="inlineStr"/>
+      <c r="BJ159" t="inlineStr">
+        <is>
+          <t>BE Product (Infrastructure)</t>
+        </is>
+      </c>
+      <c r="BK159" t="inlineStr"/>
+      <c r="BL159" t="inlineStr"/>
+      <c r="BM159" t="inlineStr"/>
+      <c r="BN159" t="inlineStr"/>
+      <c r="BO159" t="inlineStr"/>
+      <c r="BP159" t="inlineStr"/>
+      <c r="BQ159" t="inlineStr"/>
+      <c r="BR159" t="inlineStr">
+        <is>
+          <t>{owl: http://www.w3.org/2002/07/owl#}, {rdf: http://www.w3.org/1999/02/22-rdf-syntax-ns#}, {xsd: http://www.w3.org/2001/XMLSchema#}, {brot: https://w3id.org/brot#}, {foaf: http://xmlns.com/foaf/0.1/}, {rdfs: http://www.w3.org/2000/01/rdf-schema#}, {vann: http://purl.org/vocab/vann/}, {None: http://purl.org/dc/}</t>
+        </is>
+      </c>
+      <c r="BS159" t="n">
+        <v>62</v>
+      </c>
+      <c r="BT159" t="n">
+        <v>62</v>
+      </c>
+      <c r="BU159" t="n">
+        <v>14</v>
+      </c>
+      <c r="BV159" t="n">
+        <v>14</v>
+      </c>
+      <c r="BW159" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX159" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY159" t="b">
+        <v>1</v>
+      </c>
+      <c r="BZ159" t="b">
+        <v>1</v>
+      </c>
+      <c r="CA159" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB159" t="n">
+        <v>2</v>
+      </c>
+      <c r="CC159" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD159" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE159" t="b">
+        <v>0</v>
+      </c>
+      <c r="CF159" t="b">
+        <v>1</v>
+      </c>
+      <c r="CG159" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH159" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>